<commit_message>
Besiktning: Caravan Club Storsveds Camping 2026-06-06 (Excel)
</commit_message>
<xml_diff>
--- a/besiktningar/2026/Caravan_Club_Storsveds_Camping_2026-06-06.xlsx
+++ b/besiktningar/2026/Caravan_Club_Storsveds_Camping_2026-06-06.xlsx
@@ -445,7 +445,7 @@
         <v>RESULTAT</v>
       </c>
       <c r="B8" t="str">
-        <v>GODKÄND</v>
+        <v>UNDERKÄND</v>
       </c>
     </row>
     <row r="9">
@@ -453,7 +453,7 @@
         <v>Bedömda punkter</v>
       </c>
       <c r="B9">
-        <v>11</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10">
@@ -461,7 +461,7 @@
         <v>Underkända punkter (Nej)</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>